<commit_message>
fix: Jun 28 week expenses marked pending (not yet withdrawn from NBG); +€150 cleaning materials paid
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="435">
   <si>
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
@@ -713,12 +713,21 @@
     <t xml:space="preserve">Local mfr</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-06-28</t>
+    <t xml:space="preserve">2026-06-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleaning materials - Yael unit (Jun 27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upcoming</t>
   </si>
   <si>
     <t xml:space="preserve">Materials - week Jun25-28 (Yael unit completion)</t>
   </si>
   <si>
+    <t xml:space="preserve">Committed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Plumber - Yael unit completion</t>
   </si>
   <si>
@@ -737,13 +746,7 @@
     <t xml:space="preserve">Workers week Jun25-28 (Yael unit + site)</t>
   </si>
   <si>
-    <t xml:space="preserve">upcoming</t>
-  </si>
-  <si>
     <t xml:space="preserve">Electrician - 2 apts+2 storages+outdoor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Committed</t>
   </si>
   <si>
     <t xml:space="preserve">Electrical plans - submitted to authority</t>
@@ -2067,8 +2070,8 @@
         <v>10</v>
       </c>
       <c r="B10" s="9" t="n">
-        <f aca="false">'Renovation Ledger'!E134</f>
-        <v>78191.47</v>
+        <f aca="false">'Renovation Ledger'!E135</f>
+        <v>73701.47</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>11</v>
@@ -2079,8 +2082,8 @@
         <v>12</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">'Renovation Ledger'!E135</f>
-        <v>17453</v>
+        <f aca="false">'Renovation Ledger'!E136</f>
+        <v>22093</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>13</v>
@@ -2091,8 +2094,8 @@
         <v>14</v>
       </c>
       <c r="B12" s="5" t="n">
-        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E134</f>
-        <v>249900.47</v>
+        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E135</f>
+        <v>245410.47</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>15</v>
@@ -2150,7 +2153,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H137"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -5214,10 +5217,10 @@
         <v>229</v>
       </c>
       <c r="D120" s="14" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>1500</v>
+        <v>150</v>
       </c>
       <c r="F120" s="16" t="s">
         <v>34</v>
@@ -5231,19 +5234,19 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B121" s="14" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C121" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D121" s="14" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="E121" s="15" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="F121" s="16" t="s">
         <v>34</v>
@@ -5251,51 +5254,51 @@
       <c r="G121" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H121" s="17" t="s">
-        <v>36</v>
+      <c r="H121" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B122" s="14" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D122" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E122" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="F122" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="G122" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="H122" s="18" t="s">
         <v>232</v>
-      </c>
-      <c r="E122" s="15" t="n">
-        <v>250</v>
-      </c>
-      <c r="F122" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="G122" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="H122" s="17" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B123" s="14" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D123" s="14" t="s">
-        <v>44</v>
+        <v>235</v>
       </c>
       <c r="E123" s="15" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="F123" s="16" t="s">
         <v>34</v>
@@ -5303,25 +5306,25 @@
       <c r="G123" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H123" s="17" t="s">
-        <v>36</v>
+      <c r="H123" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B124" s="14" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D124" s="14" t="s">
-        <v>221</v>
+        <v>44</v>
       </c>
       <c r="E124" s="15" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F124" s="16" t="s">
         <v>34</v>
@@ -5329,25 +5332,25 @@
       <c r="G124" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H124" s="17" t="s">
-        <v>36</v>
+      <c r="H124" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B125" s="14" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D125" s="14" t="s">
-        <v>41</v>
+        <v>221</v>
       </c>
       <c r="E125" s="15" t="n">
-        <v>2600</v>
+        <v>40</v>
       </c>
       <c r="F125" s="16" t="s">
         <v>34</v>
@@ -5355,25 +5358,25 @@
       <c r="G125" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H125" s="17" t="s">
-        <v>36</v>
+      <c r="H125" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B126" s="14" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C126" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D126" s="14" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="E126" s="15" t="n">
-        <v>9500</v>
+        <v>2600</v>
       </c>
       <c r="F126" s="16" t="s">
         <v>34</v>
@@ -5382,12 +5385,12 @@
         <v>35</v>
       </c>
       <c r="H126" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B127" s="14" t="s">
         <v>42</v>
@@ -5399,21 +5402,21 @@
         <v>80</v>
       </c>
       <c r="E127" s="15" t="n">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="F127" s="16" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G127" s="16" t="s">
         <v>35</v>
       </c>
       <c r="H127" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B128" s="14" t="s">
         <v>42</v>
@@ -5425,7 +5428,7 @@
         <v>80</v>
       </c>
       <c r="E128" s="15" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="F128" s="16" t="s">
         <v>47</v>
@@ -5434,12 +5437,12 @@
         <v>35</v>
       </c>
       <c r="H128" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B129" s="14" t="s">
         <v>42</v>
@@ -5451,33 +5454,33 @@
         <v>80</v>
       </c>
       <c r="E129" s="15" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="F129" s="16" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G129" s="16" t="s">
         <v>35</v>
       </c>
       <c r="H129" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B130" s="14" t="s">
-        <v>122</v>
+        <v>42</v>
       </c>
       <c r="C130" s="14" t="s">
         <v>242</v>
       </c>
       <c r="D130" s="14" t="s">
-        <v>243</v>
+        <v>80</v>
       </c>
       <c r="E130" s="15" t="n">
-        <v>550</v>
+        <v>1000</v>
       </c>
       <c r="F130" s="16" t="s">
         <v>34</v>
@@ -5486,24 +5489,24 @@
         <v>35</v>
       </c>
       <c r="H130" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B131" s="14" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="C131" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D131" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="D131" s="14" t="s">
-        <v>162</v>
-      </c>
       <c r="E131" s="15" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="F131" s="16" t="s">
         <v>34</v>
@@ -5512,86 +5515,103 @@
         <v>35</v>
       </c>
       <c r="H131" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B132" s="14" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C132" s="14" t="s">
         <v>245</v>
       </c>
       <c r="D132" s="14" t="s">
-        <v>87</v>
+        <v>162</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>3858</v>
+        <v>600</v>
       </c>
       <c r="F132" s="16" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G132" s="16" t="s">
         <v>35</v>
       </c>
       <c r="H132" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B133" s="14" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C133" s="14" t="s">
         <v>246</v>
       </c>
       <c r="D133" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E133" s="15" t="n">
+        <v>3858</v>
+      </c>
+      <c r="F133" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="G133" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="H133" s="18" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B134" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C134" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="D134" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E133" s="15" t="n">
+      <c r="E134" s="15" t="n">
         <v>195</v>
       </c>
-      <c r="F133" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="G133" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="H133" s="18" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D134" s="19" t="s">
-        <v>247</v>
-      </c>
-      <c r="E134" s="20" t="n">
-        <f aca="false">SUMIF(H5:H133,"Paid",E5:E133)</f>
-        <v>78191.47</v>
+      <c r="F134" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="G134" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="H134" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D135" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="E135" s="21" t="n">
-        <f aca="false">SUMIF(H5:H133,"Committed",E5:E133)</f>
-        <v>17453</v>
+      <c r="E135" s="20" t="n">
+        <f aca="false">SUMIF(H5:H134,"Paid",E5:E134)</f>
+        <v>73701.47</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D136" s="22" t="s">
+      <c r="D136" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="E136" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E133,H5:H133,"Paid",G5:G133,"Yes")</f>
-        <v>76163.92</v>
+      <c r="E136" s="21" t="n">
+        <f aca="false">SUMIF(H5:H134,"Committed",E5:E134)</f>
+        <v>22093</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5599,7 +5619,16 @@
         <v>250</v>
       </c>
       <c r="E137" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E133,H5:H133,"Paid",G5:G133,"No")</f>
+        <f aca="false">SUMIFS(E5:E134,H5:H134,"Paid",G5:G134,"Yes")</f>
+        <v>71673.92</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D138" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="E138" s="23" t="n">
+        <f aca="false">SUMIFS(E5:E134,H5:H134,"Paid",G5:G134,"No")</f>
         <v>2027.55</v>
       </c>
     </row>
@@ -5635,7 +5664,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5644,7 +5673,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5653,33 +5682,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>35</v>
@@ -5687,16 +5716,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>15000</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>35</v>
@@ -5704,16 +5733,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B7" s="24" t="n">
         <v>130000</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>35</v>
@@ -5721,16 +5750,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>10000</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>35</v>
@@ -5738,16 +5767,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B9" s="24" t="n">
         <v>20000</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E9" s="17" t="s">
         <v>35</v>
@@ -5755,16 +5784,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>70000</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>35</v>
@@ -5772,16 +5801,16 @@
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B11" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>182</v>
@@ -5789,7 +5818,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B12" s="26" t="n">
         <f aca="false">SUMIF(E5:E11,"Yes",B5:B11)</f>
@@ -5798,7 +5827,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="27" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
@@ -5807,7 +5836,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -5849,7 +5878,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5858,7 +5887,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5870,10 +5899,10 @@
         <v>22</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>26</v>
@@ -5882,18 +5911,18 @@
         <v>28</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>18500</v>
@@ -5902,18 +5931,18 @@
         <v>35</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>107000</v>
@@ -5922,18 +5951,18 @@
         <v>35</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>19731</v>
@@ -5942,18 +5971,18 @@
         <v>35</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>7410</v>
@@ -5962,18 +5991,18 @@
         <v>35</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>4350</v>
@@ -5982,15 +6011,15 @@
         <v>35</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>149</v>
@@ -6002,15 +6031,15 @@
         <v>35</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>149</v>
@@ -6022,18 +6051,18 @@
         <v>35</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D12" s="24" t="n">
         <v>2490</v>
@@ -6042,18 +6071,18 @@
         <v>35</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D13" s="24" t="n">
         <v>800</v>
@@ -6062,18 +6091,18 @@
         <v>35</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D14" s="24" t="n">
         <v>520</v>
@@ -6085,13 +6114,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>680</v>
@@ -6103,13 +6132,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D16" s="24" t="n">
         <v>3000</v>
@@ -6118,15 +6147,15 @@
         <v>35</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>47</v>
@@ -6138,15 +6167,15 @@
         <v>182</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>47</v>
@@ -6158,12 +6187,12 @@
         <v>182</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="25" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">SUM(D5:D18)</f>
@@ -6172,7 +6201,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="19" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">SUMIF(E5:E18,"Yes",D5:D18)</f>
@@ -6181,7 +6210,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
@@ -6222,7 +6251,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6231,7 +6260,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6243,7 +6272,7 @@
         <v>22</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>27</v>
@@ -6252,7 +6281,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6260,7 +6289,7 @@
         <v>169</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>181</v>
@@ -6269,7 +6298,7 @@
         <v>614</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6277,7 +6306,7 @@
         <v>204</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>207</v>
@@ -6286,7 +6315,7 @@
         <v>972.55</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6294,7 +6323,7 @@
         <v>211</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>181</v>
@@ -6303,7 +6332,7 @@
         <v>286</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6311,7 +6340,7 @@
         <v>215</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>207</v>
@@ -6320,12 +6349,12 @@
         <v>155</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="19" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">SUM(D5:D8)</f>
@@ -6334,7 +6363,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -6346,7 +6375,7 @@
         <v>22</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>27</v>
@@ -6355,7 +6384,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6363,16 +6392,16 @@
         <v>215</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>972.55</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -6406,7 +6435,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6414,7 +6443,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6425,13 +6454,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6439,14 +6468,14 @@
         <v>37</v>
       </c>
       <c r="B5" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A5,'Renovation Ledger'!H5:H133,"Paid")</f>
-        <v>24550</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A5,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <v>21700</v>
       </c>
       <c r="C5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6454,14 +6483,14 @@
         <v>50</v>
       </c>
       <c r="B6" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A6,'Renovation Ledger'!H5:H133,"Paid")</f>
-        <v>25642.87</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A6,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <v>24242.87</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6469,14 +6498,14 @@
         <v>105</v>
       </c>
       <c r="B7" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A7,'Renovation Ledger'!H5:H133,"Paid")</f>
-        <v>7119</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A7,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <v>6919</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>9000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6484,14 +6513,14 @@
         <v>42</v>
       </c>
       <c r="B8" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A8,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A8,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>2325</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>11250</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6499,14 +6528,14 @@
         <v>81</v>
       </c>
       <c r="B9" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A9,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A9,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>4300</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>6000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,14 +6543,14 @@
         <v>103</v>
       </c>
       <c r="B10" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A10,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A10,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>4225</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>4500</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6529,14 +6558,14 @@
         <v>122</v>
       </c>
       <c r="B11" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A11,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A11,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>1550</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>18700</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6544,14 +6573,14 @@
         <v>31</v>
       </c>
       <c r="B12" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A12,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A12,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>2097</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6559,14 +6588,14 @@
         <v>212</v>
       </c>
       <c r="B13" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A13,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A13,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>286</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25500</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6574,14 +6603,14 @@
         <v>218</v>
       </c>
       <c r="B14" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A14,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A14,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>905</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>1000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6589,14 +6618,14 @@
         <v>76</v>
       </c>
       <c r="B15" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A15,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A15,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>3811</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>11350</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6604,14 +6633,14 @@
         <v>94</v>
       </c>
       <c r="B16" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A16,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A16,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>300</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>5000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6619,8 +6648,8 @@
         <v>70</v>
       </c>
       <c r="B17" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A17,'Renovation Ledger'!H5:H133,"Paid")</f>
-        <v>230</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A17,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <v>190</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>500</v>
@@ -6634,14 +6663,14 @@
         <v>45</v>
       </c>
       <c r="B18" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A18,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A18,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>750.6</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>500</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6649,23 +6678,23 @@
         <v>65</v>
       </c>
       <c r="B19" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E133,'Renovation Ledger'!B5:B133,A19,'Renovation Ledger'!H5:H133,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A19,'Renovation Ledger'!H5:H134,"Paid")</f>
         <v>100</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>300</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">SUM(B5:B19)</f>
-        <v>78191.47</v>
+        <v>73701.47</v>
       </c>
       <c r="C20" s="28" t="n">
         <f aca="false">SUM(C5:C19)</f>
@@ -6703,7 +6732,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6711,7 +6740,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6719,106 +6748,106 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="30" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C5" s="31" t="n">
         <v>21066.81</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C6" s="34" t="n">
         <v>230000</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="35" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>-139459.28</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="35" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>-6350</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="35" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C9" s="36" t="n">
         <v>-64730</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="35" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>-4494.92</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="35" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C11" s="36" t="n">
         <v>-711</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="35" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C12" s="36" t="n">
         <v>-104.17</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="35" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C13" s="36" t="n">
         <v>-14.5</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="29" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C14" s="37" t="n">
         <f aca="false">SUM(C5:C13)</f>
@@ -6827,7 +6856,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="29" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>35202.94</v>
@@ -6835,7 +6864,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="39" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C16" s="40" t="n">
         <f aca="false">C14-C15</f>
@@ -6844,21 +6873,21 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="29" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="41" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C19" s="42" t="n">
-        <f aca="false">'Renovation Ledger'!E136</f>
-        <v>76163.92</v>
+        <f aca="false">'Renovation Ledger'!E137</f>
+        <v>71673.92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="41" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C20" s="42" t="n">
         <v>69935.92</v>
@@ -6866,23 +6895,23 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="43" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C21" s="44" t="n">
-        <f aca="false">'Renovation Ledger'!E136-69935.92</f>
-        <v>6228</v>
+        <f aca="false">'Renovation Ledger'!E137-69935.92</f>
+        <v>1738</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="45" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="45" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="45"/>
@@ -6921,7 +6950,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6930,7 +6959,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6939,189 +6968,189 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: project update 2026-07-06 -- week Jun29-Jul5 expenses (€4,300) approved, SikaGrout 340 structural cost flagged (~€20K est.), Antonis fee renegotiated
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Renovation Ledger'!E135</f>
+        <f>'Renovation Ledger'!E140</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>'Renovation Ledger'!E136</f>
+        <f>'Renovation Ledger'!E141</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E135</f>
+        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E140</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -818,7 +818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I138"/>
+  <dimension ref="A1:I143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6386,26 +6386,26 @@
     <row r="127">
       <c r="A127" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B127" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C127" s="14" t="inlineStr">
         <is>
-          <t>Electrician - 2 apts+2 storages+outdoor</t>
+          <t>Sand and gravel - week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D127" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E127" s="15" t="n">
-        <v>9500</v>
+        <v>150</v>
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
@@ -6417,40 +6417,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H127" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I127" s="14" t="inlineStr"/>
+      <c r="H127" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I127" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Fuel</t>
         </is>
       </c>
       <c r="C128" s="14" t="inlineStr">
         <is>
-          <t>Electrical plans - submitted to authority</t>
+          <t>Fuel - concrete mixers week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D128" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Gas station</t>
         </is>
       </c>
       <c r="E128" s="15" t="n">
-        <v>1000</v>
+        <v>40</v>
       </c>
       <c r="F128" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G128" s="16" t="inlineStr">
@@ -6458,40 +6462,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H128" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I128" s="14" t="inlineStr"/>
+      <c r="H128" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I128" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B129" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>Three-phase meter (Kobi's name)</t>
+          <t>Steel reinforcement - wall bond beams above door openings</t>
         </is>
       </c>
       <c r="D129" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E129" s="15" t="n">
-        <v>750</v>
+        <v>400</v>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G129" s="16" t="inlineStr">
@@ -6499,36 +6507,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H129" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I129" s="14" t="inlineStr"/>
+      <c r="H129" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I129" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B130" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>Electrician advance - 130m piping reimb.</t>
+          <t>Kairis - column reinforcement steel, cement, resin anchors</t>
         </is>
       </c>
       <c r="D130" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Kairis</t>
         </is>
       </c>
       <c r="E130" s="15" t="n">
-        <v>1000</v>
+        <v>1800</v>
       </c>
       <c r="F130" s="16" t="inlineStr">
         <is>
@@ -6540,36 +6552,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H130" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I130" s="14" t="inlineStr"/>
+      <c r="H130" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B131" s="14" t="inlineStr">
         <is>
-          <t>Windows/Iron</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="C131" s="14" t="inlineStr">
         <is>
-          <t>Metalworker - small storage door+window</t>
+          <t>Workers wages - week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D131" s="14" t="inlineStr">
         <is>
-          <t>Metalworker</t>
+          <t>Workers</t>
         </is>
       </c>
       <c r="E131" s="15" t="n">
-        <v>550</v>
+        <v>1910</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -6581,36 +6597,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H131" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I131" s="14" t="inlineStr"/>
+      <c r="H131" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I131" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>Site Works</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C132" s="14" t="inlineStr">
         <is>
-          <t>Excavator - road compaction (60t roller)</t>
+          <t>Electrician - 2 apts+2 storages+outdoor</t>
         </is>
       </c>
       <c r="D132" s="14" t="inlineStr">
         <is>
-          <t>Excavator</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E132" s="15" t="n">
-        <v>600</v>
+        <v>9500</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -6632,26 +6652,26 @@
     <row r="133">
       <c r="A133" s="14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B133" s="14" t="inlineStr">
         <is>
-          <t>Legal/Admin</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C133" s="14" t="inlineStr">
         <is>
-          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+          <t>Electrical plans - submitted to authority</t>
         </is>
       </c>
       <c r="D133" s="14" t="inlineStr">
         <is>
-          <t>EFKA</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E133" s="15" t="n">
-        <v>3858</v>
+        <v>1000</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
@@ -6673,85 +6693,290 @@
     <row r="134">
       <c r="A134" s="14" t="inlineStr">
         <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B134" s="14" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="C134" s="14" t="inlineStr">
+        <is>
+          <t>Three-phase meter (Kobi's name)</t>
+        </is>
+      </c>
+      <c r="D134" s="14" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="E134" s="15" t="n">
+        <v>750</v>
+      </c>
+      <c r="F134" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G134" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H134" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I134" s="14" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B135" s="14" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="C135" s="14" t="inlineStr">
+        <is>
+          <t>Electrician advance - 130m piping reimb.</t>
+        </is>
+      </c>
+      <c r="D135" s="14" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="E135" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F135" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G135" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H135" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I135" s="14" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B136" s="14" t="inlineStr">
+        <is>
+          <t>Windows/Iron</t>
+        </is>
+      </c>
+      <c r="C136" s="14" t="inlineStr">
+        <is>
+          <t>Metalworker - small storage door+window</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>Metalworker</t>
+        </is>
+      </c>
+      <c r="E136" s="15" t="n">
+        <v>550</v>
+      </c>
+      <c r="F136" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G136" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H136" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I136" s="14" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B137" s="14" t="inlineStr">
+        <is>
+          <t>Site Works</t>
+        </is>
+      </c>
+      <c r="C137" s="14" t="inlineStr">
+        <is>
+          <t>Excavator - road compaction (60t roller)</t>
+        </is>
+      </c>
+      <c r="D137" s="14" t="inlineStr">
+        <is>
+          <t>Excavator</t>
+        </is>
+      </c>
+      <c r="E137" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="F137" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G137" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H137" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I137" s="14" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B138" s="14" t="inlineStr">
+        <is>
+          <t>Legal/Admin</t>
+        </is>
+      </c>
+      <c r="C138" s="14" t="inlineStr">
+        <is>
+          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>EFKA</t>
+        </is>
+      </c>
+      <c r="E138" s="15" t="n">
+        <v>3858</v>
+      </c>
+      <c r="F138" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G138" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H138" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I138" s="14" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="inlineStr">
+        <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B134" s="14" t="inlineStr">
+      <c r="B139" s="14" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="C134" s="14" t="inlineStr">
+      <c r="C139" s="14" t="inlineStr">
         <is>
           <t>Kairis - remaining balance</t>
         </is>
       </c>
-      <c r="D134" s="14" t="inlineStr">
+      <c r="D139" s="14" t="inlineStr">
         <is>
           <t>Kairis</t>
         </is>
       </c>
-      <c r="E134" s="15" t="n">
+      <c r="E139" s="15" t="n">
         <v>195</v>
       </c>
-      <c r="F134" s="16" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="G134" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H134" s="18" t="inlineStr">
+      <c r="F139" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G139" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H139" s="18" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>
       </c>
-      <c r="I134" s="14" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="D135" s="19" t="inlineStr">
+      <c r="I139" s="14" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="D140" s="19" t="inlineStr">
         <is>
           <t>PAID — total</t>
         </is>
       </c>
-      <c r="E135" s="20">
-        <f>SUMIF(H5:H134,"Paid",E5:E134)</f>
+      <c r="E140" s="20">
+        <f>SUMIF(H5:H139,"Paid",E5:E139)</f>
         <v/>
       </c>
     </row>
-    <row r="136">
-      <c r="D136" s="19" t="inlineStr">
+    <row r="141">
+      <c r="D141" s="19" t="inlineStr">
         <is>
           <t>COMMITTED (approved, unpaid)</t>
         </is>
       </c>
-      <c r="E136" s="21">
-        <f>SUMIF(H5:H134,"Committed",E5:E134)</f>
+      <c r="E141" s="21">
+        <f>SUMIF(H5:H139,"Committed",E5:E139)</f>
         <v/>
       </c>
     </row>
-    <row r="137">
-      <c r="D137" s="22" t="inlineStr">
+    <row r="142">
+      <c r="D142" s="22" t="inlineStr">
         <is>
           <t>PAID — from NBG (cash/transfer)</t>
         </is>
       </c>
-      <c r="E137" s="23">
-        <f>SUMIFS(E5:E134,H5:H134,"Paid",G5:G134,"Yes")</f>
+      <c r="E142" s="23">
+        <f>SUMIFS(E5:E139,H5:H139,"Paid",G5:G139,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="138">
-      <c r="D138" s="22" t="inlineStr">
+    <row r="143">
+      <c r="D143" s="22" t="inlineStr">
         <is>
           <t>PAID — outside NBG (Wise/card)</t>
         </is>
       </c>
-      <c r="E138" s="23">
-        <f>SUMIFS(E5:E134,H5:H134,"Paid",G5:G134,"No")</f>
+      <c r="E143" s="23">
+        <f>SUMIFS(E5:E139,H5:H139,"Paid",G5:G139,"No")</f>
         <v/>
       </c>
     </row>
@@ -7841,7 +8066,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A5,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A5,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n">
@@ -7860,7 +8085,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A6,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A6,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n">
@@ -7879,7 +8104,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A7,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A7,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n">
@@ -7898,7 +8123,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A8,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A8,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C8" s="24" t="n">
@@ -7917,7 +8142,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A9,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A9,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n">
@@ -7936,7 +8161,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A10,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A10,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n">
@@ -7955,7 +8180,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A11,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A11,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C11" s="24" t="n">
@@ -7974,7 +8199,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A12,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A12,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C12" s="24" t="n">
@@ -7993,7 +8218,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A13,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A13,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C13" s="24" t="n">
@@ -8012,7 +8237,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A14,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A14,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C14" s="24" t="n">
@@ -8031,7 +8256,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A15,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A15,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C15" s="24" t="n">
@@ -8050,7 +8275,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A16,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A16,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C16" s="24" t="n">
@@ -8069,7 +8294,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A17,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A17,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C17" s="24" t="n">
@@ -8088,7 +8313,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A18,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A18,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C18" s="24" t="n">
@@ -8107,7 +8332,7 @@
         </is>
       </c>
       <c r="B19" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E134,'Renovation Ledger'!B5:B134,A19,'Renovation Ledger'!H5:H134,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A19,'Renovation Ledger'!H5:H139,"Paid")</f>
         <v/>
       </c>
       <c r="C19" s="24" t="n">
@@ -8353,7 +8578,7 @@
         </is>
       </c>
       <c r="C19" s="41">
-        <f>'Renovation Ledger'!E137</f>
+        <f>'Renovation Ledger'!E142</f>
         <v/>
       </c>
     </row>
@@ -8374,7 +8599,7 @@
         </is>
       </c>
       <c r="C21" s="43">
-        <f>'Renovation Ledger'!E137-69935.92</f>
+        <f>'Renovation Ledger'!E142-69935.92</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: project update 2026-07-07 -- precision fix: split week Jun29-Jul5 batch into Committed (EUR4,300 approved) + Paid (EUR3,000 actually withdrawn), avoids overstating cash-out
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Renovation Ledger'!E140</f>
+        <f>'Renovation Ledger'!E141</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>'Renovation Ledger'!E141</f>
+        <f>'Renovation Ledger'!E142</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E140</f>
+        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E141</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -818,7 +818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6116,26 +6116,26 @@
     <row r="121">
       <c r="A121" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B121" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>Materials - week Jun25-28 (Yael unit completion)</t>
+          <t>Cash withdrawal - partial funding for week Jun29-Jul5 batch (item-level allocation TBC)</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>Vicky (cash withdrawal)</t>
         </is>
       </c>
       <c r="E121" s="15" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
@@ -6154,33 +6154,33 @@
       </c>
       <c r="I121" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B122" s="14" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Plumber - Yael unit completion</t>
+          <t>Sand and gravel - week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>Plumber</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E122" s="15" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F122" s="16" t="inlineStr">
         <is>
@@ -6192,40 +6192,36 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H122" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I122" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H122" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I122" s="14" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B123" s="14" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Fuel</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>Carpenter - Yael unit (bedside tables/countertop/door)</t>
+          <t>Fuel - concrete mixers week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>Carpenter</t>
+          <t>Gas station</t>
         </is>
       </c>
       <c r="E123" s="15" t="n">
-        <v>250</v>
+        <v>40</v>
       </c>
       <c r="F123" s="16" t="inlineStr">
         <is>
@@ -6237,21 +6233,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H123" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I123" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H123" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I123" s="14" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B124" s="14" t="inlineStr">
@@ -6261,7 +6253,7 @@
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>Marble for shower - Yael unit</t>
+          <t>Steel reinforcement - wall bond beams above door openings</t>
         </is>
       </c>
       <c r="D124" s="14" t="inlineStr">
@@ -6270,7 +6262,7 @@
         </is>
       </c>
       <c r="E124" s="15" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="F124" s="16" t="inlineStr">
         <is>
@@ -6282,40 +6274,36 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H124" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I124" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H124" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I124" s="14" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B125" s="14" t="inlineStr">
         <is>
-          <t>Fuel</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C125" s="14" t="inlineStr">
         <is>
-          <t>Site fuel week Jun25-28</t>
+          <t>Kairis - column reinforcement steel, cement, resin anchors</t>
         </is>
       </c>
       <c r="D125" s="14" t="inlineStr">
         <is>
-          <t>Vicky</t>
+          <t>Kairis</t>
         </is>
       </c>
       <c r="E125" s="15" t="n">
-        <v>40</v>
+        <v>1800</v>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
@@ -6327,21 +6315,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H125" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I125" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H125" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I125" s="14" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B126" s="14" t="inlineStr">
@@ -6351,7 +6335,7 @@
       </c>
       <c r="C126" s="14" t="inlineStr">
         <is>
-          <t>Workers week Jun25-28 (Yael unit + site)</t>
+          <t>Workers wages - week Jun29-Jul5</t>
         </is>
       </c>
       <c r="D126" s="14" t="inlineStr">
@@ -6360,7 +6344,7 @@
         </is>
       </c>
       <c r="E126" s="15" t="n">
-        <v>2600</v>
+        <v>1910</v>
       </c>
       <c r="F126" s="16" t="inlineStr">
         <is>
@@ -6372,21 +6356,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H126" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I126" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H126" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I126" s="14" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B127" s="14" t="inlineStr">
@@ -6396,16 +6376,16 @@
       </c>
       <c r="C127" s="14" t="inlineStr">
         <is>
-          <t>Sand and gravel - week Jun29-Jul5</t>
+          <t>Materials - week Jun25-28 (Yael unit completion)</t>
         </is>
       </c>
       <c r="D127" s="14" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Kairis</t>
         </is>
       </c>
       <c r="E127" s="15" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
@@ -6424,33 +6404,33 @@
       </c>
       <c r="I127" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>Fuel</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="C128" s="14" t="inlineStr">
         <is>
-          <t>Fuel - concrete mixers week Jun29-Jul5</t>
+          <t>Plumber - Yael unit completion</t>
         </is>
       </c>
       <c r="D128" s="14" t="inlineStr">
         <is>
-          <t>Gas station</t>
+          <t>Plumber</t>
         </is>
       </c>
       <c r="E128" s="15" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="F128" s="16" t="inlineStr">
         <is>
@@ -6469,33 +6449,33 @@
       </c>
       <c r="I128" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B129" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>Steel reinforcement - wall bond beams above door openings</t>
+          <t>Carpenter - Yael unit (bedside tables/countertop/door)</t>
         </is>
       </c>
       <c r="D129" s="14" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Carpenter</t>
         </is>
       </c>
       <c r="E129" s="15" t="n">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
@@ -6514,14 +6494,14 @@
       </c>
       <c r="I129" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B130" s="14" t="inlineStr">
@@ -6531,16 +6511,16 @@
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>Kairis - column reinforcement steel, cement, resin anchors</t>
+          <t>Marble for shower - Yael unit</t>
         </is>
       </c>
       <c r="D130" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E130" s="15" t="n">
-        <v>1800</v>
+        <v>50</v>
       </c>
       <c r="F130" s="16" t="inlineStr">
         <is>
@@ -6559,33 +6539,33 @@
       </c>
       <c r="I130" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B131" s="14" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Fuel</t>
         </is>
       </c>
       <c r="C131" s="14" t="inlineStr">
         <is>
-          <t>Workers wages - week Jun29-Jul5</t>
+          <t>Site fuel week Jun25-28</t>
         </is>
       </c>
       <c r="D131" s="14" t="inlineStr">
         <is>
-          <t>Workers</t>
+          <t>Vicky</t>
         </is>
       </c>
       <c r="E131" s="15" t="n">
-        <v>1910</v>
+        <v>40</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -6604,33 +6584,33 @@
       </c>
       <c r="I131" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="C132" s="14" t="inlineStr">
         <is>
-          <t>Electrician - 2 apts+2 storages+outdoor</t>
+          <t>Workers week Jun25-28 (Yael unit + site)</t>
         </is>
       </c>
       <c r="D132" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Workers</t>
         </is>
       </c>
       <c r="E132" s="15" t="n">
-        <v>9500</v>
+        <v>2600</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -6642,12 +6622,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H132" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I132" s="14" t="inlineStr"/>
+      <c r="H132" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I132" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="14" t="inlineStr">
@@ -6662,7 +6646,7 @@
       </c>
       <c r="C133" s="14" t="inlineStr">
         <is>
-          <t>Electrical plans - submitted to authority</t>
+          <t>Electrician - 2 apts+2 storages+outdoor</t>
         </is>
       </c>
       <c r="D133" s="14" t="inlineStr">
@@ -6671,11 +6655,11 @@
         </is>
       </c>
       <c r="E133" s="15" t="n">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G133" s="16" t="inlineStr">
@@ -6703,7 +6687,7 @@
       </c>
       <c r="C134" s="14" t="inlineStr">
         <is>
-          <t>Three-phase meter (Kobi's name)</t>
+          <t>Electrical plans - submitted to authority</t>
         </is>
       </c>
       <c r="D134" s="14" t="inlineStr">
@@ -6712,7 +6696,7 @@
         </is>
       </c>
       <c r="E134" s="15" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="F134" s="16" t="inlineStr">
         <is>
@@ -6744,7 +6728,7 @@
       </c>
       <c r="C135" s="14" t="inlineStr">
         <is>
-          <t>Electrician advance - 130m piping reimb.</t>
+          <t>Three-phase meter (Kobi's name)</t>
         </is>
       </c>
       <c r="D135" s="14" t="inlineStr">
@@ -6753,11 +6737,11 @@
         </is>
       </c>
       <c r="E135" s="15" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="F135" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G135" s="16" t="inlineStr">
@@ -6780,21 +6764,21 @@
       </c>
       <c r="B136" s="14" t="inlineStr">
         <is>
-          <t>Windows/Iron</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C136" s="14" t="inlineStr">
         <is>
-          <t>Metalworker - small storage door+window</t>
+          <t>Electrician advance - 130m piping reimb.</t>
         </is>
       </c>
       <c r="D136" s="14" t="inlineStr">
         <is>
-          <t>Metalworker</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E136" s="15" t="n">
-        <v>550</v>
+        <v>1000</v>
       </c>
       <c r="F136" s="16" t="inlineStr">
         <is>
@@ -6816,26 +6800,26 @@
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B137" s="14" t="inlineStr">
         <is>
-          <t>Site Works</t>
+          <t>Windows/Iron</t>
         </is>
       </c>
       <c r="C137" s="14" t="inlineStr">
         <is>
-          <t>Excavator - road compaction (60t roller)</t>
+          <t>Metalworker - small storage door+window</t>
         </is>
       </c>
       <c r="D137" s="14" t="inlineStr">
         <is>
-          <t>Excavator</t>
+          <t>Metalworker</t>
         </is>
       </c>
       <c r="E137" s="15" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
@@ -6857,30 +6841,30 @@
     <row r="138">
       <c r="A138" s="14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B138" s="14" t="inlineStr">
         <is>
-          <t>Legal/Admin</t>
+          <t>Site Works</t>
         </is>
       </c>
       <c r="C138" s="14" t="inlineStr">
         <is>
-          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+          <t>Excavator - road compaction (60t roller)</t>
         </is>
       </c>
       <c r="D138" s="14" t="inlineStr">
         <is>
-          <t>EFKA</t>
+          <t>Excavator</t>
         </is>
       </c>
       <c r="E138" s="15" t="n">
-        <v>3858</v>
+        <v>600</v>
       </c>
       <c r="F138" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G138" s="16" t="inlineStr">
@@ -6898,85 +6882,126 @@
     <row r="139">
       <c r="A139" s="14" t="inlineStr">
         <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B139" s="14" t="inlineStr">
+        <is>
+          <t>Legal/Admin</t>
+        </is>
+      </c>
+      <c r="C139" s="14" t="inlineStr">
+        <is>
+          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>EFKA</t>
+        </is>
+      </c>
+      <c r="E139" s="15" t="n">
+        <v>3858</v>
+      </c>
+      <c r="F139" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G139" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H139" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I139" s="14" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="inlineStr">
+        <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B139" s="14" t="inlineStr">
+      <c r="B140" s="14" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="C139" s="14" t="inlineStr">
+      <c r="C140" s="14" t="inlineStr">
         <is>
           <t>Kairis - remaining balance</t>
         </is>
       </c>
-      <c r="D139" s="14" t="inlineStr">
+      <c r="D140" s="14" t="inlineStr">
         <is>
           <t>Kairis</t>
         </is>
       </c>
-      <c r="E139" s="15" t="n">
+      <c r="E140" s="15" t="n">
         <v>195</v>
       </c>
-      <c r="F139" s="16" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="G139" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H139" s="18" t="inlineStr">
+      <c r="F140" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G140" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H140" s="18" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>
       </c>
-      <c r="I139" s="14" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="D140" s="19" t="inlineStr">
-        <is>
-          <t>PAID — total</t>
-        </is>
-      </c>
-      <c r="E140" s="20">
-        <f>SUMIF(H5:H139,"Paid",E5:E139)</f>
-        <v/>
-      </c>
+      <c r="I140" s="14" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="D141" s="19" t="inlineStr">
         <is>
+          <t>PAID — total</t>
+        </is>
+      </c>
+      <c r="E141" s="20">
+        <f>SUMIF(H5:H140,"Paid",E5:E140)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="D142" s="19" t="inlineStr">
+        <is>
           <t>COMMITTED (approved, unpaid)</t>
         </is>
       </c>
-      <c r="E141" s="21">
-        <f>SUMIF(H5:H139,"Committed",E5:E139)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="142">
-      <c r="D142" s="22" t="inlineStr">
-        <is>
-          <t>PAID — from NBG (cash/transfer)</t>
-        </is>
-      </c>
-      <c r="E142" s="23">
-        <f>SUMIFS(E5:E139,H5:H139,"Paid",G5:G139,"Yes")</f>
+      <c r="E142" s="21">
+        <f>SUMIF(H5:H140,"Committed",E5:E140)</f>
         <v/>
       </c>
     </row>
     <row r="143">
       <c r="D143" s="22" t="inlineStr">
         <is>
+          <t>PAID — from NBG (cash/transfer)</t>
+        </is>
+      </c>
+      <c r="E143" s="23">
+        <f>SUMIFS(E5:E140,H5:H140,"Paid",G5:G140,"Yes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="D144" s="22" t="inlineStr">
+        <is>
           <t>PAID — outside NBG (Wise/card)</t>
         </is>
       </c>
-      <c r="E143" s="23">
-        <f>SUMIFS(E5:E139,H5:H139,"Paid",G5:G139,"No")</f>
+      <c r="E144" s="23">
+        <f>SUMIFS(E5:E140,H5:H140,"Paid",G5:G140,"No")</f>
         <v/>
       </c>
     </row>
@@ -8066,7 +8091,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A5,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A5,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n">
@@ -8085,7 +8110,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A6,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A6,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n">
@@ -8104,7 +8129,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A7,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A7,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n">
@@ -8123,7 +8148,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A8,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A8,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C8" s="24" t="n">
@@ -8142,7 +8167,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A9,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A9,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n">
@@ -8161,7 +8186,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A10,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A10,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n">
@@ -8180,7 +8205,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A11,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A11,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C11" s="24" t="n">
@@ -8199,7 +8224,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A12,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A12,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C12" s="24" t="n">
@@ -8218,7 +8243,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A13,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A13,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C13" s="24" t="n">
@@ -8237,7 +8262,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A14,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A14,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C14" s="24" t="n">
@@ -8256,7 +8281,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A15,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A15,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C15" s="24" t="n">
@@ -8275,7 +8300,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A16,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A16,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C16" s="24" t="n">
@@ -8294,7 +8319,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A17,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A17,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C17" s="24" t="n">
@@ -8313,7 +8338,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A18,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A18,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C18" s="24" t="n">
@@ -8332,7 +8357,7 @@
         </is>
       </c>
       <c r="B19" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E139,'Renovation Ledger'!B5:B139,A19,'Renovation Ledger'!H5:H139,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E140,'Renovation Ledger'!B5:B140,A19,'Renovation Ledger'!H5:H140,"Paid")</f>
         <v/>
       </c>
       <c r="C19" s="24" t="n">
@@ -8578,7 +8603,7 @@
         </is>
       </c>
       <c r="C19" s="41">
-        <f>'Renovation Ledger'!E142</f>
+        <f>'Renovation Ledger'!E143</f>
         <v/>
       </c>
     </row>
@@ -8599,7 +8624,7 @@
         </is>
       </c>
       <c r="C21" s="43">
-        <f>'Renovation Ledger'!E142-69935.92</f>
+        <f>'Renovation Ledger'!E143-69935.92</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: project update 2026-07-11 -- fixed stale NBG balance in balance sheet, reconciled to EUR23,505.02 (EUR907.92 gap flagged)
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="460">
   <si>
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Financial ground truth. Currency: EUR. Last updated 25 Jun 2026. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
+    <t xml:space="preserve">Financial ground truth. Currency: EUR. Last updated 2026-07-11. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
   </si>
   <si>
     <t xml:space="preserve">FUNDING &amp; POSITION</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Current NBG balance</t>
   </si>
   <si>
-    <t xml:space="preserve">Per official NBG statement, 25-Jun-2026</t>
+    <t xml:space="preserve">Reported 2026-07-11 (see Reconciliation &gt; Rolling Bridge for the residual check)</t>
   </si>
   <si>
     <t xml:space="preserve">RENOVATION</t>
@@ -1247,6 +1247,30 @@
     <t xml:space="preserve">The small ledger-vs-statement difference is cash float (cash withdrawn vs spent timing). ATM withdrawals are exact; renovation cash expenses are reconstructed weekly estimates.</t>
   </si>
   <si>
+    <t xml:space="preserve">ROLLING BRIDGE — since last full statement (2026-06-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening — statement closing balance (2026-06-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Deposits since (dynamic — recalculates as new transfers are added)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Renovation paid from NBG since (dynamic — recalculates as new expenses are added)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Computed balance (bridge)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reported balance (2026-07-11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residual (bridge − reported)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A residual here is expected cash-float/timing (ATM withdrawals vs itemized weekly reconstructions), or spending not yet reported to Kobi -- see Flags &amp; Dedup. It is NOT unexplained/missing money unless it grows unexpectedly large or keeps widening.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flags &amp; De-duplication Log</t>
   </si>
   <si>
@@ -1371,6 +1395,18 @@
   </si>
   <si>
     <t xml:space="preserve">Pay/confirm; then it moves to Paid.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR907.92 residual — rolling bridge (25-Jun to 11-Jul)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kobi reported the current NBG balance as EUR23,505.02 on 11-Jul-2026. The ledger only accounts for EUR10,790 in NBG-paid cash-out since the 25-Jun statement (EUR35,202.94), projecting EUR24,412.94 -- EUR907.92 more than reported. Consistent with the known cash-float pattern (round ATM withdrawals vs itemized weekly reconstructions) but could also be spending Vicky hasn't reported yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ask Vicky to confirm — either an ATM withdrawal that ran ahead of itemized expenses, or a payment not yet reported in the WhatsApp group.</t>
   </si>
 </sst>
 </file>
@@ -1382,7 +1418,7 @@
     <numFmt numFmtId="165" formatCode="\€#,##0"/>
     <numFmt numFmtId="166" formatCode="\€#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1497,8 +1533,16 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1538,6 +1582,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFD6E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor rgb="FFD6E0F0"/>
       </patternFill>
     </fill>
@@ -1591,7 +1641,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1780,6 +1830,22 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1830,7 +1896,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -2089,12 +2155,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>35202.94</v>
+        <v>23505.02</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>8</v>
@@ -7342,7 +7408,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -7537,12 +7603,80 @@
       <c r="C24" s="46"/>
       <c r="D24" s="46"/>
     </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="47" t="s">
+        <v>406</v>
+      </c>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="42" t="s">
+        <v>407</v>
+      </c>
+      <c r="C27" s="43" t="n">
+        <v>35202.94</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="42" t="s">
+        <v>408</v>
+      </c>
+      <c r="C28" s="43" t="n">
+        <f aca="false">SUMPRODUCT(('Funding (NBG Deposits)'!A5:A11&gt;"2026-06-25")*('Funding (NBG Deposits)'!E5:E11="Yes")*'Funding (NBG Deposits)'!B5:B11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="42" t="s">
+        <v>409</v>
+      </c>
+      <c r="C29" s="43" t="n">
+        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I141&gt;"2026-06-25")*('Renovation Ledger'!H5:H141="Paid")*('Renovation Ledger'!G5:G141="Yes")*'Renovation Ledger'!E5:E141)</f>
+        <v>10790</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="30" t="s">
+        <v>410</v>
+      </c>
+      <c r="C30" s="48" t="n">
+        <f aca="false">C27+C28-C29</f>
+        <v>24412.94</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="30" t="s">
+        <v>411</v>
+      </c>
+      <c r="C31" s="49" t="n">
+        <v>23505.02</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="40" t="s">
+        <v>412</v>
+      </c>
+      <c r="C32" s="50" t="n">
+        <f aca="false">C30-C31</f>
+        <v>907.920000000002</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="28" t="s">
+        <v>413</v>
+      </c>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B33:D33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7559,7 +7693,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -7571,7 +7705,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7580,7 +7714,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7589,189 +7723,206 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C7" s="15" t="s">
+        <v>431</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>423</v>
       </c>
-      <c r="D7" s="18" t="s">
-        <v>415</v>
-      </c>
       <c r="E7" s="15" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>447</v>
+        <v>455</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>458</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>454</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: project update 2026-07-11 -- Kairis total confirmed EUR13,730 (EUR5,240 debt + EUR7,740 order + EUR750), Committed now EUR31,183
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="462">
   <si>
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
@@ -807,6 +807,12 @@
   </si>
   <si>
     <t xml:space="preserve">Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kairis - additional item per Vicky Jul11 running-total correction (detail unspecified, confirms total EUR13,730)</t>
   </si>
   <si>
     <t xml:space="preserve">PAID — total</t>
@@ -2179,7 +2185,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="10" t="n">
-        <f aca="false">'Renovation Ledger'!E142</f>
+        <f aca="false">'Renovation Ledger'!E144</f>
         <v>84341.47</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -2191,8 +2197,8 @@
         <v>12</v>
       </c>
       <c r="B11" s="11" t="n">
-        <f aca="false">'Renovation Ledger'!E143</f>
-        <v>25193</v>
+        <f aca="false">'Renovation Ledger'!E145</f>
+        <v>31183</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>13</v>
@@ -2203,7 +2209,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E142</f>
+        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E144</f>
         <v>256050.47</v>
       </c>
       <c r="C12" s="7" t="s">
@@ -2262,7 +2268,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="13"/>
@@ -6283,39 +6289,93 @@
       </c>
       <c r="I141" s="15"/>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D142" s="20" t="s">
+    <row r="142" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="B142" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C142" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="E142" s="21" t="n">
-        <f aca="false">SUMIF(H5:H141,"Paid",E5:E141)</f>
+      <c r="D142" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E142" s="16" t="n">
+        <v>5240</v>
+      </c>
+      <c r="F142" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="G142" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="I142" s="15"/>
+    </row>
+    <row r="143" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="B143" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C143" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="D143" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E143" s="16" t="n">
+        <v>750</v>
+      </c>
+      <c r="F143" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="G143" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H143" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="I143" s="15"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D144" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="E144" s="21" t="n">
+        <f aca="false">SUMIF(H5:H143,"Paid",E5:E143)</f>
         <v>84341.47</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D143" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="E143" s="22" t="n">
-        <f aca="false">SUMIF(H5:H141,"Committed",E5:E141)</f>
-        <v>25193</v>
-      </c>
-    </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D144" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="E144" s="24" t="n">
-        <f aca="false">SUMIFS(E5:E141,H5:H141,"Paid",G5:G141,"Yes")</f>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D145" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="E145" s="22" t="n">
+        <f aca="false">SUMIF(H5:H143,"Committed",E5:E143)</f>
+        <v>31183</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D146" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="E146" s="24" t="n">
+        <f aca="false">SUMIFS(E5:E143,H5:H143,"Paid",G5:G143,"Yes")</f>
         <v>82313.92</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D145" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="E145" s="24" t="n">
-        <f aca="false">SUMIFS(E5:E141,H5:H141,"Paid",G5:G141,"No")</f>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D147" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="E147" s="24" t="n">
+        <f aca="false">SUMIFS(E5:E143,H5:H143,"Paid",G5:G143,"No")</f>
         <v>2027.55</v>
       </c>
     </row>
@@ -6351,7 +6411,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6360,7 +6420,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6369,33 +6429,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B5" s="25" t="n">
         <v>25000</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>36</v>
@@ -6403,16 +6463,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B6" s="25" t="n">
         <v>15000</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E6" s="18" t="s">
         <v>36</v>
@@ -6420,16 +6480,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B7" s="25" t="n">
         <v>130000</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>36</v>
@@ -6437,16 +6497,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>10000</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>36</v>
@@ -6454,16 +6514,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B9" s="25" t="n">
         <v>20000</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>36</v>
@@ -6471,16 +6531,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B10" s="25" t="n">
         <v>70000</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>36</v>
@@ -6488,16 +6548,16 @@
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B11" s="25" t="n">
         <v>2000</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E11" s="19" t="s">
         <v>183</v>
@@ -6505,7 +6565,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B12" s="27" t="n">
         <f aca="false">SUMIF(E5:E11,"Yes",B5:B11)</f>
@@ -6514,7 +6574,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -6523,7 +6583,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -6565,7 +6625,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6574,7 +6634,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6583,13 +6643,13 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>26</v>
@@ -6598,18 +6658,18 @@
         <v>28</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D5" s="25" t="n">
         <v>18500</v>
@@ -6618,18 +6678,18 @@
         <v>36</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D6" s="25" t="n">
         <v>107000</v>
@@ -6638,18 +6698,18 @@
         <v>36</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>303</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>307</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>301</v>
       </c>
       <c r="D7" s="25" t="n">
         <v>19731</v>
@@ -6658,18 +6718,18 @@
         <v>36</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D8" s="25" t="n">
         <v>7410</v>
@@ -6678,18 +6738,18 @@
         <v>36</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D9" s="25" t="n">
         <v>4350</v>
@@ -6698,15 +6758,15 @@
         <v>36</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>150</v>
@@ -6718,15 +6778,15 @@
         <v>36</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>150</v>
@@ -6738,18 +6798,18 @@
         <v>36</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D12" s="25" t="n">
         <v>2490</v>
@@ -6758,18 +6818,18 @@
         <v>36</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D13" s="25" t="n">
         <v>800</v>
@@ -6778,18 +6838,18 @@
         <v>36</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>330</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>327</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>328</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>325</v>
       </c>
       <c r="D14" s="25" t="n">
         <v>520</v>
@@ -6801,13 +6861,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D15" s="25" t="n">
         <v>680</v>
@@ -6819,13 +6879,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D16" s="25" t="n">
         <v>3000</v>
@@ -6834,15 +6894,15 @@
         <v>36</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C17" s="15" t="s">
         <v>48</v>
@@ -6854,15 +6914,15 @@
         <v>183</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>48</v>
@@ -6874,12 +6934,12 @@
         <v>183</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="26" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D19" s="27" t="n">
         <f aca="false">SUM(D5:D18)</f>
@@ -6888,7 +6948,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="20" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D20" s="29" t="n">
         <f aca="false">SUMIF(E5:E18,"Yes",D5:D18)</f>
@@ -6897,7 +6957,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -6938,7 +6998,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6947,7 +7007,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6956,10 +7016,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>27</v>
@@ -6968,7 +7028,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6976,7 +7036,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>182</v>
@@ -6985,7 +7045,7 @@
         <v>614</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6993,7 +7053,7 @@
         <v>205</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>208</v>
@@ -7002,7 +7062,7 @@
         <v>972.55</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7010,7 +7070,7 @@
         <v>212</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>182</v>
@@ -7019,7 +7079,7 @@
         <v>286</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7027,7 +7087,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>208</v>
@@ -7036,12 +7096,12 @@
         <v>155</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="20" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D9" s="21" t="n">
         <f aca="false">SUM(D5:D8)</f>
@@ -7050,7 +7110,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -7059,10 +7119,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>27</v>
@@ -7071,7 +7131,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7079,16 +7139,16 @@
         <v>216</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>972.55</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -7122,7 +7182,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7130,7 +7190,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7141,13 +7201,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7155,14 +7215,14 @@
         <v>38</v>
       </c>
       <c r="B5" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A5,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A5,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>26460</v>
       </c>
       <c r="C5" s="25" t="n">
         <v>25000</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,14 +7230,14 @@
         <v>51</v>
       </c>
       <c r="B6" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A6,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A6,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>29842.87</v>
       </c>
       <c r="C6" s="25" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7185,14 +7245,14 @@
         <v>106</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A7,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A7,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>7119</v>
       </c>
       <c r="C7" s="25" t="n">
         <v>9000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7200,14 +7260,14 @@
         <v>43</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A8,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A8,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>2325</v>
       </c>
       <c r="C8" s="25" t="n">
         <v>11250</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7215,14 +7275,14 @@
         <v>82</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A9,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A9,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>4300</v>
       </c>
       <c r="C9" s="25" t="n">
         <v>6000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7230,14 +7290,14 @@
         <v>104</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A10,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A10,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>4225</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>4500</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7245,14 +7305,14 @@
         <v>123</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A11,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A11,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>1550</v>
       </c>
       <c r="C11" s="25" t="n">
         <v>18700</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7260,14 +7320,14 @@
         <v>32</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A12,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A12,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>2097</v>
       </c>
       <c r="C12" s="25" t="n">
         <v>2000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7275,14 +7335,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A13,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A13,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>286</v>
       </c>
       <c r="C13" s="25" t="n">
         <v>25500</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7290,14 +7350,14 @@
         <v>219</v>
       </c>
       <c r="B14" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A14,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A14,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>905</v>
       </c>
       <c r="C14" s="25" t="n">
         <v>1000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7305,14 +7365,14 @@
         <v>77</v>
       </c>
       <c r="B15" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A15,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A15,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>3811</v>
       </c>
       <c r="C15" s="25" t="n">
         <v>11350</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7320,14 +7380,14 @@
         <v>95</v>
       </c>
       <c r="B16" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A16,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A16,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>300</v>
       </c>
       <c r="C16" s="25" t="n">
         <v>5000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7335,7 +7395,7 @@
         <v>71</v>
       </c>
       <c r="B17" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A17,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A17,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>270</v>
       </c>
       <c r="C17" s="25" t="n">
@@ -7350,14 +7410,14 @@
         <v>46</v>
       </c>
       <c r="B18" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A18,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A18,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>750.6</v>
       </c>
       <c r="C18" s="25" t="n">
         <v>500</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7365,19 +7425,19 @@
         <v>66</v>
       </c>
       <c r="B19" s="16" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E141,'Renovation Ledger'!B5:B141,A19,'Renovation Ledger'!H5:H141,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E143,'Renovation Ledger'!B5:B143,A19,'Renovation Ledger'!H5:H143,"Paid")</f>
         <v>100</v>
       </c>
       <c r="C19" s="25" t="n">
         <v>300</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B20" s="21" t="n">
         <f aca="false">SUM(B5:B19)</f>
@@ -7419,7 +7479,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7427,7 +7487,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7435,106 +7495,106 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="31" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C5" s="32" t="n">
         <v>21066.81</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C6" s="35" t="n">
         <v>230000</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="36" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C7" s="37" t="n">
         <v>-139459.28</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="36" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C8" s="37" t="n">
         <v>-6350</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="36" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C9" s="37" t="n">
         <v>-64730</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="36" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C10" s="37" t="n">
         <v>-4494.92</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="36" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C11" s="37" t="n">
         <v>-711</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="36" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C12" s="37" t="n">
         <v>-104.17</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="36" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C13" s="37" t="n">
         <v>-14.5</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="30" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C14" s="38" t="n">
         <f aca="false">SUM(C5:C13)</f>
@@ -7543,7 +7603,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="30" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C15" s="39" t="n">
         <v>35202.94</v>
@@ -7551,7 +7611,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="40" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C16" s="41" t="n">
         <f aca="false">C14-C15</f>
@@ -7560,21 +7620,21 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="30" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="42" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C19" s="43" t="n">
-        <f aca="false">'Renovation Ledger'!E144</f>
+        <f aca="false">'Renovation Ledger'!E146</f>
         <v>82313.92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="42" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C20" s="43" t="n">
         <v>69935.92</v>
@@ -7582,37 +7642,37 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="44" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C21" s="45" t="n">
-        <f aca="false">'Renovation Ledger'!E144-69935.92</f>
+        <f aca="false">'Renovation Ledger'!E146-69935.92</f>
         <v>12378</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="46" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C23" s="46"/>
       <c r="D23" s="46"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="46" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C24" s="46"/>
       <c r="D24" s="46"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="47" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C26" s="47"/>
       <c r="D26" s="47"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="42" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C27" s="43" t="n">
         <v>35202.94</v>
@@ -7620,7 +7680,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="42" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C28" s="43" t="n">
         <f aca="false">SUMPRODUCT(('Funding (NBG Deposits)'!A5:A11&gt;"2026-06-25")*('Funding (NBG Deposits)'!E5:E11="Yes")*'Funding (NBG Deposits)'!B5:B11)</f>
@@ -7629,16 +7689,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="42" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C29" s="43" t="n">
-        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I141&gt;"2026-06-25")*('Renovation Ledger'!H5:H141="Paid")*('Renovation Ledger'!G5:G141="Yes")*'Renovation Ledger'!E5:E141)</f>
+        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I143&gt;"2026-06-25")*('Renovation Ledger'!H5:H143="Paid")*('Renovation Ledger'!G5:G143="Yes")*'Renovation Ledger'!E5:E143)</f>
         <v>10790</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C30" s="48" t="n">
         <f aca="false">C27+C28-C29</f>
@@ -7647,7 +7707,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C31" s="49" t="n">
         <v>23505.02</v>
@@ -7655,7 +7715,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="40" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C32" s="50" t="n">
         <f aca="false">C30-C31</f>
@@ -7664,7 +7724,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="28" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C33" s="28"/>
       <c r="D33" s="28"/>
@@ -7705,7 +7765,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7714,7 +7774,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7723,206 +7783,206 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>428</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>429</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>426</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>427</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>423</v>
-      </c>
       <c r="E6" s="15" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
+        <v>458</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>460</v>
+      </c>
+      <c r="D15" s="19" t="s">
         <v>456</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>457</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>458</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>454</v>
-      </c>
       <c r="E15" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: project update 2026-07-20 -- Vicky's delayed week Jul13-19 report (€985 labor, insurance cleared to pay, heat delay on SikaGrout)
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Renovation Ledger'!E145</f>
+        <f>'Renovation Ledger'!E148</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>'Renovation Ledger'!E146</f>
+        <f>'Renovation Ledger'!E149</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E145</f>
+        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E148</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6452,26 +6452,26 @@
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="C128" s="14" t="inlineStr">
         <is>
-          <t>Materials - week Jun25-28 (Yael unit completion)</t>
+          <t>Workers wages Mon-Wed - week Jul13-19</t>
         </is>
       </c>
       <c r="D128" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>Workers</t>
         </is>
       </c>
       <c r="E128" s="15" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="F128" s="16" t="inlineStr">
         <is>
@@ -6483,40 +6483,36 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H128" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I128" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H128" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I128" s="14" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B129" s="14" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>Plumber - Yael unit completion</t>
+          <t>Concrete mixer - week Jul13-19</t>
         </is>
       </c>
       <c r="D129" s="14" t="inlineStr">
         <is>
-          <t>Plumber</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="E129" s="15" t="n">
-        <v>200</v>
+        <v>20</v>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
@@ -6528,40 +6524,36 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H129" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I129" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H129" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I129" s="14" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B130" s="14" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>Carpenter - Yael unit (bedside tables/countertop/door)</t>
+          <t>Binding wire and steel-tying materials - week Jul13-19</t>
         </is>
       </c>
       <c r="D130" s="14" t="inlineStr">
         <is>
-          <t>Carpenter</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E130" s="15" t="n">
-        <v>250</v>
+        <v>65</v>
       </c>
       <c r="F130" s="16" t="inlineStr">
         <is>
@@ -6573,16 +6565,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H130" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I130" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
+      <c r="H130" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
@@ -6597,16 +6585,16 @@
       </c>
       <c r="C131" s="14" t="inlineStr">
         <is>
-          <t>Marble for shower - Yael unit</t>
+          <t>Materials - week Jun25-28 (Yael unit completion)</t>
         </is>
       </c>
       <c r="D131" s="14" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Kairis</t>
         </is>
       </c>
       <c r="E131" s="15" t="n">
-        <v>50</v>
+        <v>1500</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -6637,21 +6625,21 @@
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>Fuel</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="C132" s="14" t="inlineStr">
         <is>
-          <t>Site fuel week Jun25-28</t>
+          <t>Plumber - Yael unit completion</t>
         </is>
       </c>
       <c r="D132" s="14" t="inlineStr">
         <is>
-          <t>Vicky</t>
+          <t>Plumber</t>
         </is>
       </c>
       <c r="E132" s="15" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -6687,16 +6675,16 @@
       </c>
       <c r="C133" s="14" t="inlineStr">
         <is>
-          <t>Workers week Jun25-28 (Yael unit + site)</t>
+          <t>Carpenter - Yael unit (bedside tables/countertop/door)</t>
         </is>
       </c>
       <c r="D133" s="14" t="inlineStr">
         <is>
-          <t>Workers</t>
+          <t>Carpenter</t>
         </is>
       </c>
       <c r="E133" s="15" t="n">
-        <v>2600</v>
+        <v>250</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
@@ -6722,26 +6710,26 @@
     <row r="134">
       <c r="A134" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B134" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C134" s="14" t="inlineStr">
         <is>
-          <t>Electrician - 2 apts+2 storages+outdoor</t>
+          <t>Marble for shower - Yael unit</t>
         </is>
       </c>
       <c r="D134" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="E134" s="15" t="n">
-        <v>9500</v>
+        <v>50</v>
       </c>
       <c r="F134" s="16" t="inlineStr">
         <is>
@@ -6753,40 +6741,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H134" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I134" s="14" t="inlineStr"/>
+      <c r="H134" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I134" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B135" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Fuel</t>
         </is>
       </c>
       <c r="C135" s="14" t="inlineStr">
         <is>
-          <t>Electrical plans - submitted to authority</t>
+          <t>Site fuel week Jun25-28</t>
         </is>
       </c>
       <c r="D135" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Vicky</t>
         </is>
       </c>
       <c r="E135" s="15" t="n">
-        <v>1000</v>
+        <v>40</v>
       </c>
       <c r="F135" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G135" s="16" t="inlineStr">
@@ -6794,40 +6786,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H135" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I135" s="14" t="inlineStr"/>
+      <c r="H135" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I135" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="14" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B136" s="14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Labour</t>
         </is>
       </c>
       <c r="C136" s="14" t="inlineStr">
         <is>
-          <t>Three-phase meter (Kobi's name)</t>
+          <t>Workers week Jun25-28 (Yael unit + site)</t>
         </is>
       </c>
       <c r="D136" s="14" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Workers</t>
         </is>
       </c>
       <c r="E136" s="15" t="n">
-        <v>750</v>
+        <v>2600</v>
       </c>
       <c r="F136" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G136" s="16" t="inlineStr">
@@ -6835,12 +6831,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H136" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I136" s="14" t="inlineStr"/>
+      <c r="H136" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I136" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
@@ -6855,7 +6855,7 @@
       </c>
       <c r="C137" s="14" t="inlineStr">
         <is>
-          <t>Electrician advance - 130m piping reimb.</t>
+          <t>Electrician - 2 apts+2 storages+outdoor</t>
         </is>
       </c>
       <c r="D137" s="14" t="inlineStr">
@@ -6864,7 +6864,7 @@
         </is>
       </c>
       <c r="E137" s="15" t="n">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
@@ -6891,25 +6891,25 @@
       </c>
       <c r="B138" s="14" t="inlineStr">
         <is>
-          <t>Windows/Iron</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C138" s="14" t="inlineStr">
         <is>
-          <t>Metalworker - small storage door+window</t>
+          <t>Electrical plans - submitted to authority</t>
         </is>
       </c>
       <c r="D138" s="14" t="inlineStr">
         <is>
-          <t>Metalworker</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E138" s="15" t="n">
-        <v>550</v>
+        <v>1000</v>
       </c>
       <c r="F138" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G138" s="16" t="inlineStr">
@@ -6927,30 +6927,30 @@
     <row r="139">
       <c r="A139" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B139" s="14" t="inlineStr">
         <is>
-          <t>Site Works</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C139" s="14" t="inlineStr">
         <is>
-          <t>Excavator - road compaction (60t roller)</t>
+          <t>Three-phase meter (Kobi's name)</t>
         </is>
       </c>
       <c r="D139" s="14" t="inlineStr">
         <is>
-          <t>Excavator</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E139" s="15" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="F139" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G139" s="16" t="inlineStr">
@@ -6968,30 +6968,30 @@
     <row r="140">
       <c r="A140" s="14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B140" s="14" t="inlineStr">
         <is>
-          <t>Legal/Admin</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C140" s="14" t="inlineStr">
         <is>
-          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+          <t>Electrician advance - 130m piping reimb.</t>
         </is>
       </c>
       <c r="D140" s="14" t="inlineStr">
         <is>
-          <t>EFKA</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="E140" s="15" t="n">
-        <v>3858</v>
+        <v>1000</v>
       </c>
       <c r="F140" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G140" s="16" t="inlineStr">
@@ -7009,26 +7009,26 @@
     <row r="141">
       <c r="A141" s="14" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B141" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Windows/Iron</t>
         </is>
       </c>
       <c r="C141" s="14" t="inlineStr">
         <is>
-          <t>Kairis - remaining balance</t>
+          <t>Metalworker - small storage door+window</t>
         </is>
       </c>
       <c r="D141" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>Metalworker</t>
         </is>
       </c>
       <c r="E141" s="15" t="n">
-        <v>195</v>
+        <v>550</v>
       </c>
       <c r="F141" s="16" t="inlineStr">
         <is>
@@ -7050,26 +7050,26 @@
     <row r="142">
       <c r="A142" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B142" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Site Works</t>
         </is>
       </c>
       <c r="C142" s="14" t="inlineStr">
         <is>
-          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+          <t>Excavator - road compaction (60t roller)</t>
         </is>
       </c>
       <c r="D142" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>Excavator</t>
         </is>
       </c>
       <c r="E142" s="15" t="n">
-        <v>7740</v>
+        <v>600</v>
       </c>
       <c r="F142" s="16" t="inlineStr">
         <is>
@@ -7091,30 +7091,30 @@
     <row r="143">
       <c r="A143" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B143" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Legal/Admin</t>
         </is>
       </c>
       <c r="C143" s="14" t="inlineStr">
         <is>
-          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
         </is>
       </c>
       <c r="D143" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>EFKA</t>
         </is>
       </c>
       <c r="E143" s="15" t="n">
-        <v>5240</v>
+        <v>3858</v>
       </c>
       <c r="F143" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G143" s="16" t="inlineStr">
@@ -7132,85 +7132,208 @@
     <row r="144">
       <c r="A144" s="14" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B144" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C144" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - remaining balance</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E144" s="15" t="n">
+        <v>195</v>
+      </c>
+      <c r="F144" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G144" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H144" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I144" s="14" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="14" t="inlineStr">
+        <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B144" s="14" t="inlineStr">
+      <c r="B145" s="14" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="C144" s="14" t="inlineStr">
+      <c r="C145" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+        </is>
+      </c>
+      <c r="D145" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E145" s="15" t="n">
+        <v>7740</v>
+      </c>
+      <c r="F145" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G145" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H145" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I145" s="14" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B146" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C146" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+        </is>
+      </c>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E146" s="15" t="n">
+        <v>5240</v>
+      </c>
+      <c r="F146" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G146" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H146" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I146" s="14" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B147" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C147" s="14" t="inlineStr">
         <is>
           <t>Kairis - additional item per Vicky Jul11 running-total correction (detail unspecified, confirms total EUR13,730)</t>
         </is>
       </c>
-      <c r="D144" s="14" t="inlineStr">
+      <c r="D147" s="14" t="inlineStr">
         <is>
           <t>Kairis</t>
         </is>
       </c>
-      <c r="E144" s="15" t="n">
+      <c r="E147" s="15" t="n">
         <v>750</v>
       </c>
-      <c r="F144" s="16" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="G144" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H144" s="18" t="inlineStr">
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G147" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H147" s="18" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>
       </c>
-      <c r="I144" s="14" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="D145" s="19" t="inlineStr">
+      <c r="I147" s="14" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="D148" s="19" t="inlineStr">
         <is>
           <t>PAID — total</t>
         </is>
       </c>
-      <c r="E145" s="20">
-        <f>SUMIF(H5:H144,"Paid",E5:E144)</f>
+      <c r="E148" s="20">
+        <f>SUMIF(H5:H147,"Paid",E5:E147)</f>
         <v/>
       </c>
     </row>
-    <row r="146">
-      <c r="D146" s="19" t="inlineStr">
+    <row r="149">
+      <c r="D149" s="19" t="inlineStr">
         <is>
           <t>COMMITTED (approved, unpaid)</t>
         </is>
       </c>
-      <c r="E146" s="21">
-        <f>SUMIF(H5:H144,"Committed",E5:E144)</f>
+      <c r="E149" s="21">
+        <f>SUMIF(H5:H147,"Committed",E5:E147)</f>
         <v/>
       </c>
     </row>
-    <row r="147">
-      <c r="D147" s="22" t="inlineStr">
+    <row r="150">
+      <c r="D150" s="22" t="inlineStr">
         <is>
           <t>PAID — from NBG (cash/transfer)</t>
         </is>
       </c>
-      <c r="E147" s="23">
-        <f>SUMIFS(E5:E144,H5:H144,"Paid",G5:G144,"Yes")</f>
+      <c r="E150" s="23">
+        <f>SUMIFS(E5:E147,H5:H147,"Paid",G5:G147,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="148">
-      <c r="D148" s="22" t="inlineStr">
+    <row r="151">
+      <c r="D151" s="22" t="inlineStr">
         <is>
           <t>PAID — outside NBG (Wise/card)</t>
         </is>
       </c>
-      <c r="E148" s="23">
-        <f>SUMIFS(E5:E144,H5:H144,"Paid",G5:G144,"No")</f>
+      <c r="E151" s="23">
+        <f>SUMIFS(E5:E147,H5:H147,"Paid",G5:G147,"No")</f>
         <v/>
       </c>
     </row>
@@ -8325,7 +8448,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A5,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A5,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n">
@@ -8344,7 +8467,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A6,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A6,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n">
@@ -8363,7 +8486,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A7,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A7,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n">
@@ -8382,7 +8505,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A8,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A8,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C8" s="24" t="n">
@@ -8401,7 +8524,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A9,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A9,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n">
@@ -8420,7 +8543,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A10,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A10,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n">
@@ -8439,7 +8562,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A11,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A11,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C11" s="24" t="n">
@@ -8458,7 +8581,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A12,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A12,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C12" s="24" t="n">
@@ -8477,7 +8600,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A13,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A13,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C13" s="24" t="n">
@@ -8496,7 +8619,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A14,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A14,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C14" s="24" t="n">
@@ -8515,7 +8638,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A15,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A15,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C15" s="24" t="n">
@@ -8534,7 +8657,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A16,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A16,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C16" s="24" t="n">
@@ -8553,7 +8676,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A17,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A17,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C17" s="24" t="n">
@@ -8572,7 +8695,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A18,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A18,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C18" s="24" t="n">
@@ -8591,7 +8714,7 @@
         </is>
       </c>
       <c r="B19" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E144,'Renovation Ledger'!B5:B144,A19,'Renovation Ledger'!H5:H144,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A19,'Renovation Ledger'!H5:H147,"Paid")</f>
         <v/>
       </c>
       <c r="C19" s="24" t="n">
@@ -8837,7 +8960,7 @@
         </is>
       </c>
       <c r="C19" s="41">
-        <f>'Renovation Ledger'!E147</f>
+        <f>'Renovation Ledger'!E150</f>
         <v/>
       </c>
     </row>
@@ -8858,7 +8981,7 @@
         </is>
       </c>
       <c r="C21" s="43">
-        <f>'Renovation Ledger'!E147-69935.92</f>
+        <f>'Renovation Ledger'!E150-69935.92</f>
         <v/>
       </c>
     </row>
@@ -8911,7 +9034,7 @@
         </is>
       </c>
       <c r="C29" s="41">
-        <f>SUMPRODUCT(('Renovation Ledger'!I5:I144&gt;"2026-06-25")*('Renovation Ledger'!H5:H144="Paid")*('Renovation Ledger'!G5:G144="Yes")*'Renovation Ledger'!E5:E144)</f>
+        <f>SUMPRODUCT(('Renovation Ledger'!I5:I147&gt;"2026-06-25")*('Renovation Ledger'!H5:H147="Paid")*('Renovation Ledger'!G5:G147="Yes")*'Renovation Ledger'!E5:E147)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: project update 2026-07-20 evening -- EUR3,000 withdrawal reconciled (labor+Kairis+insurance), alt mix discussion logged
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Renovation Ledger'!E148</f>
+        <f>'Renovation Ledger'!E150</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>'Renovation Ledger'!E149</f>
+        <f>'Renovation Ledger'!E151</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E148</f>
+        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E150</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6483,12 +6483,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H128" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I128" s="14" t="inlineStr"/>
+      <c r="H128" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I128" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="inlineStr">
@@ -6524,12 +6528,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H129" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I129" s="14" t="inlineStr"/>
+      <c r="H129" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I129" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
@@ -6565,12 +6573,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H130" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I130" s="14" t="inlineStr"/>
+      <c r="H130" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
@@ -7091,7 +7103,7 @@
     <row r="143">
       <c r="A143" s="14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B143" s="14" t="inlineStr">
@@ -7101,7 +7113,7 @@
       </c>
       <c r="C143" s="14" t="inlineStr">
         <is>
-          <t>Worker insurance Apr-Jun (€1,286 x3)</t>
+          <t>Worker insurance Apr-Jun - partial payment</t>
         </is>
       </c>
       <c r="D143" s="14" t="inlineStr">
@@ -7110,11 +7122,11 @@
         </is>
       </c>
       <c r="E143" s="15" t="n">
-        <v>3858</v>
+        <v>1865</v>
       </c>
       <c r="F143" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G143" s="16" t="inlineStr">
@@ -7122,40 +7134,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H143" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I143" s="14" t="inlineStr"/>
+      <c r="H143" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I143" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="14" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B144" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Legal/Admin</t>
         </is>
       </c>
       <c r="C144" s="14" t="inlineStr">
         <is>
-          <t>Kairis - remaining balance</t>
+          <t>Worker insurance Apr-Jun - remaining balance</t>
         </is>
       </c>
       <c r="D144" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>EFKA</t>
         </is>
       </c>
       <c r="E144" s="15" t="n">
-        <v>195</v>
+        <v>1993</v>
       </c>
       <c r="F144" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G144" s="16" t="inlineStr">
@@ -7173,7 +7189,7 @@
     <row r="145">
       <c r="A145" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B145" s="14" t="inlineStr">
@@ -7183,7 +7199,7 @@
       </c>
       <c r="C145" s="14" t="inlineStr">
         <is>
-          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+          <t>Kairis - partial payment (ATM shortfall from last week)</t>
         </is>
       </c>
       <c r="D145" s="14" t="inlineStr">
@@ -7192,7 +7208,7 @@
         </is>
       </c>
       <c r="E145" s="15" t="n">
-        <v>7740</v>
+        <v>150</v>
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
@@ -7204,17 +7220,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H145" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I145" s="14" t="inlineStr"/>
+      <c r="H145" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I145" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B146" s="14" t="inlineStr">
@@ -7224,7 +7244,7 @@
       </c>
       <c r="C146" s="14" t="inlineStr">
         <is>
-          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+          <t>Kairis - remaining balance</t>
         </is>
       </c>
       <c r="D146" s="14" t="inlineStr">
@@ -7233,7 +7253,7 @@
         </is>
       </c>
       <c r="E146" s="15" t="n">
-        <v>5240</v>
+        <v>45</v>
       </c>
       <c r="F146" s="16" t="inlineStr">
         <is>
@@ -7265,75 +7285,157 @@
       </c>
       <c r="C147" s="14" t="inlineStr">
         <is>
+          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+        </is>
+      </c>
+      <c r="D147" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E147" s="15" t="n">
+        <v>7740</v>
+      </c>
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G147" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H147" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I147" s="14" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B148" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+        </is>
+      </c>
+      <c r="D148" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E148" s="15" t="n">
+        <v>5240</v>
+      </c>
+      <c r="F148" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G148" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H148" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I148" s="14" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B149" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C149" s="14" t="inlineStr">
+        <is>
           <t>Kairis - additional item per Vicky Jul11 running-total correction (detail unspecified, confirms total EUR13,730)</t>
         </is>
       </c>
-      <c r="D147" s="14" t="inlineStr">
+      <c r="D149" s="14" t="inlineStr">
         <is>
           <t>Kairis</t>
         </is>
       </c>
-      <c r="E147" s="15" t="n">
+      <c r="E149" s="15" t="n">
         <v>750</v>
       </c>
-      <c r="F147" s="16" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="G147" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H147" s="18" t="inlineStr">
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G149" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H149" s="18" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>
       </c>
-      <c r="I147" s="14" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="D148" s="19" t="inlineStr">
+      <c r="I149" s="14" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="D150" s="19" t="inlineStr">
         <is>
           <t>PAID — total</t>
         </is>
       </c>
-      <c r="E148" s="20">
-        <f>SUMIF(H5:H147,"Paid",E5:E147)</f>
+      <c r="E150" s="20">
+        <f>SUMIF(H5:H149,"Paid",E5:E149)</f>
         <v/>
       </c>
     </row>
-    <row r="149">
-      <c r="D149" s="19" t="inlineStr">
+    <row r="151">
+      <c r="D151" s="19" t="inlineStr">
         <is>
           <t>COMMITTED (approved, unpaid)</t>
         </is>
       </c>
-      <c r="E149" s="21">
-        <f>SUMIF(H5:H147,"Committed",E5:E147)</f>
+      <c r="E151" s="21">
+        <f>SUMIF(H5:H149,"Committed",E5:E149)</f>
         <v/>
       </c>
     </row>
-    <row r="150">
-      <c r="D150" s="22" t="inlineStr">
+    <row r="152">
+      <c r="D152" s="22" t="inlineStr">
         <is>
           <t>PAID — from NBG (cash/transfer)</t>
         </is>
       </c>
-      <c r="E150" s="23">
-        <f>SUMIFS(E5:E147,H5:H147,"Paid",G5:G147,"Yes")</f>
+      <c r="E152" s="23">
+        <f>SUMIFS(E5:E149,H5:H149,"Paid",G5:G149,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="151">
-      <c r="D151" s="22" t="inlineStr">
+    <row r="153">
+      <c r="D153" s="22" t="inlineStr">
         <is>
           <t>PAID — outside NBG (Wise/card)</t>
         </is>
       </c>
-      <c r="E151" s="23">
-        <f>SUMIFS(E5:E147,H5:H147,"Paid",G5:G147,"No")</f>
+      <c r="E153" s="23">
+        <f>SUMIFS(E5:E149,H5:H149,"Paid",G5:G149,"No")</f>
         <v/>
       </c>
     </row>
@@ -8448,7 +8550,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A5,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A5,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n">
@@ -8467,7 +8569,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A6,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A6,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n">
@@ -8486,7 +8588,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A7,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A7,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n">
@@ -8505,7 +8607,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A8,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A8,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C8" s="24" t="n">
@@ -8524,7 +8626,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A9,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A9,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n">
@@ -8543,7 +8645,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A10,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A10,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n">
@@ -8562,7 +8664,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A11,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A11,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C11" s="24" t="n">
@@ -8581,7 +8683,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A12,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A12,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C12" s="24" t="n">
@@ -8600,7 +8702,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A13,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A13,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C13" s="24" t="n">
@@ -8619,7 +8721,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A14,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A14,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C14" s="24" t="n">
@@ -8638,7 +8740,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A15,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A15,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C15" s="24" t="n">
@@ -8657,7 +8759,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A16,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A16,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C16" s="24" t="n">
@@ -8676,7 +8778,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A17,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A17,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C17" s="24" t="n">
@@ -8695,7 +8797,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A18,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A18,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C18" s="24" t="n">
@@ -8714,7 +8816,7 @@
         </is>
       </c>
       <c r="B19" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E147,'Renovation Ledger'!B5:B147,A19,'Renovation Ledger'!H5:H147,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A19,'Renovation Ledger'!H5:H149,"Paid")</f>
         <v/>
       </c>
       <c r="C19" s="24" t="n">
@@ -8960,7 +9062,7 @@
         </is>
       </c>
       <c r="C19" s="41">
-        <f>'Renovation Ledger'!E150</f>
+        <f>'Renovation Ledger'!E152</f>
         <v/>
       </c>
     </row>
@@ -8981,7 +9083,7 @@
         </is>
       </c>
       <c r="C21" s="43">
-        <f>'Renovation Ledger'!E150-69935.92</f>
+        <f>'Renovation Ledger'!E152-69935.92</f>
         <v/>
       </c>
     </row>
@@ -9034,7 +9136,7 @@
         </is>
       </c>
       <c r="C29" s="41">
-        <f>SUMPRODUCT(('Renovation Ledger'!I5:I147&gt;"2026-06-25")*('Renovation Ledger'!H5:H147="Paid")*('Renovation Ledger'!G5:G147="Yes")*'Renovation Ledger'!E5:E147)</f>
+        <f>SUMPRODUCT(('Renovation Ledger'!I5:I149&gt;"2026-06-25")*('Renovation Ledger'!H5:H149="Paid")*('Renovation Ledger'!G5:G149="Yes")*'Renovation Ledger'!E5:E149)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: project update 2026-07-21 -- NBG balance 65505, second withdrawal (insurance nearly settled, Kairis 1000), reconciliation gap flagged 768
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -677,7 +677,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Financial ground truth. Currency: EUR. Last updated 2026-07-13. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
+          <t>Financial ground truth. Currency: EUR. Last updated 2026-07-21. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
         </is>
       </c>
     </row>
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>70000</v>
+        <v>65505</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Reported 2026-07-13 (see Reconciliation &gt; Rolling Bridge for the residual check)</t>
+          <t>Reported 2026-07-21 (see Reconciliation &gt; Rolling Bridge for the residual check)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Renovation Ledger'!E150</f>
+        <f>'Renovation Ledger'!E152</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>'Renovation Ledger'!E151</f>
+        <f>'Renovation Ledger'!E153</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E150</f>
+        <f>'Property Acquisition 2025'!D19+'Renovation Ledger'!E152</f>
         <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I153"/>
+  <dimension ref="A1:I155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7148,7 +7148,7 @@
     <row r="144">
       <c r="A144" s="14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B144" s="14" t="inlineStr">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C144" s="14" t="inlineStr">
         <is>
-          <t>Worker insurance Apr-Jun - remaining balance</t>
+          <t>Worker insurance Apr-Jun - second partial payment</t>
         </is>
       </c>
       <c r="D144" s="14" t="inlineStr">
@@ -7167,11 +7167,11 @@
         </is>
       </c>
       <c r="E144" s="15" t="n">
-        <v>1993</v>
+        <v>1990</v>
       </c>
       <c r="F144" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cash</t>
         </is>
       </c>
       <c r="G144" s="16" t="inlineStr">
@@ -7179,40 +7179,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H144" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I144" s="14" t="inlineStr"/>
+      <c r="H144" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I144" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="14" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B145" s="14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Legal/Admin</t>
         </is>
       </c>
       <c r="C145" s="14" t="inlineStr">
         <is>
-          <t>Kairis - partial payment (ATM shortfall from last week)</t>
+          <t>Worker insurance Apr-Jun - remaining balance</t>
         </is>
       </c>
       <c r="D145" s="14" t="inlineStr">
         <is>
-          <t>Kairis</t>
+          <t>EFKA</t>
         </is>
       </c>
       <c r="E145" s="15" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G145" s="16" t="inlineStr">
@@ -7220,21 +7224,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H145" s="17" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="I145" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
+      <c r="H145" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I145" s="14" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="14" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B146" s="14" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="C146" s="14" t="inlineStr">
         <is>
-          <t>Kairis - remaining balance</t>
+          <t>Kairis - partial payment (ATM shortfall from last week)</t>
         </is>
       </c>
       <c r="D146" s="14" t="inlineStr">
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="E146" s="15" t="n">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="F146" s="16" t="inlineStr">
         <is>
@@ -7265,17 +7265,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H146" s="18" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
-      </c>
-      <c r="I146" s="14" t="inlineStr"/>
+      <c r="H146" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I146" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B147" s="14" t="inlineStr">
@@ -7285,7 +7289,7 @@
       </c>
       <c r="C147" s="14" t="inlineStr">
         <is>
-          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
+          <t>Kairis - remaining balance</t>
         </is>
       </c>
       <c r="D147" s="14" t="inlineStr">
@@ -7294,7 +7298,7 @@
         </is>
       </c>
       <c r="E147" s="15" t="n">
-        <v>7740</v>
+        <v>45</v>
       </c>
       <c r="F147" s="16" t="inlineStr">
         <is>
@@ -7326,7 +7330,7 @@
       </c>
       <c r="C148" s="14" t="inlineStr">
         <is>
-          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10)</t>
+          <t>Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed</t>
         </is>
       </c>
       <c r="D148" s="14" t="inlineStr">
@@ -7335,7 +7339,7 @@
         </is>
       </c>
       <c r="E148" s="15" t="n">
-        <v>5240</v>
+        <v>7740</v>
       </c>
       <c r="F148" s="16" t="inlineStr">
         <is>
@@ -7357,85 +7361,171 @@
     <row r="149">
       <c r="A149" s="14" t="inlineStr">
         <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B149" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C149" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - partial payment toward column/beam debt</t>
+        </is>
+      </c>
+      <c r="D149" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E149" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G149" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H149" s="17" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I149" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="inlineStr">
+        <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B149" s="14" t="inlineStr">
+      <c r="B150" s="14" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="C149" s="14" t="inlineStr">
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t>Kairis - outstanding debt for column/beam materials received this week (EUR3,420+EUR3,530=EUR6,940, minus EUR1,700 already paid Jul10, minus EUR1,000 paid Jul21)</t>
+        </is>
+      </c>
+      <c r="D150" s="14" t="inlineStr">
+        <is>
+          <t>Kairis</t>
+        </is>
+      </c>
+      <c r="E150" s="15" t="n">
+        <v>4240</v>
+      </c>
+      <c r="F150" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G150" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H150" s="18" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="I150" s="14" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B151" s="14" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="C151" s="14" t="inlineStr">
         <is>
           <t>Kairis - additional item per Vicky Jul11 running-total correction (detail unspecified, confirms total EUR13,730)</t>
         </is>
       </c>
-      <c r="D149" s="14" t="inlineStr">
+      <c r="D151" s="14" t="inlineStr">
         <is>
           <t>Kairis</t>
         </is>
       </c>
-      <c r="E149" s="15" t="n">
+      <c r="E151" s="15" t="n">
         <v>750</v>
       </c>
-      <c r="F149" s="16" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="G149" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H149" s="18" t="inlineStr">
+      <c r="F151" s="16" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="G151" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H151" s="18" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>
       </c>
-      <c r="I149" s="14" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="D150" s="19" t="inlineStr">
+      <c r="I151" s="14" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="D152" s="19" t="inlineStr">
         <is>
           <t>PAID — total</t>
         </is>
       </c>
-      <c r="E150" s="20">
-        <f>SUMIF(H5:H149,"Paid",E5:E149)</f>
+      <c r="E152" s="20">
+        <f>SUMIF(H5:H151,"Paid",E5:E151)</f>
         <v/>
       </c>
     </row>
-    <row r="151">
-      <c r="D151" s="19" t="inlineStr">
+    <row r="153">
+      <c r="D153" s="19" t="inlineStr">
         <is>
           <t>COMMITTED (approved, unpaid)</t>
         </is>
       </c>
-      <c r="E151" s="21">
-        <f>SUMIF(H5:H149,"Committed",E5:E149)</f>
+      <c r="E153" s="21">
+        <f>SUMIF(H5:H151,"Committed",E5:E151)</f>
         <v/>
       </c>
     </row>
-    <row r="152">
-      <c r="D152" s="22" t="inlineStr">
+    <row r="154">
+      <c r="D154" s="22" t="inlineStr">
         <is>
           <t>PAID — from NBG (cash/transfer)</t>
         </is>
       </c>
-      <c r="E152" s="23">
-        <f>SUMIFS(E5:E149,H5:H149,"Paid",G5:G149,"Yes")</f>
+      <c r="E154" s="23">
+        <f>SUMIFS(E5:E151,H5:H151,"Paid",G5:G151,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="153">
-      <c r="D153" s="22" t="inlineStr">
+    <row r="155">
+      <c r="D155" s="22" t="inlineStr">
         <is>
           <t>PAID — outside NBG (Wise/card)</t>
         </is>
       </c>
-      <c r="E153" s="23">
-        <f>SUMIFS(E5:E149,H5:H149,"Paid",G5:G149,"No")</f>
+      <c r="E155" s="23">
+        <f>SUMIFS(E5:E151,H5:H151,"Paid",G5:G151,"No")</f>
         <v/>
       </c>
     </row>
@@ -8550,7 +8640,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A5,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A5,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n">
@@ -8569,7 +8659,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A6,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A6,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n">
@@ -8588,7 +8678,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A7,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A7,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n">
@@ -8607,7 +8697,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A8,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A8,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C8" s="24" t="n">
@@ -8626,7 +8716,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A9,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A9,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n">
@@ -8645,7 +8735,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A10,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A10,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n">
@@ -8664,7 +8754,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A11,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A11,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C11" s="24" t="n">
@@ -8683,7 +8773,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A12,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A12,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C12" s="24" t="n">
@@ -8702,7 +8792,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A13,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A13,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C13" s="24" t="n">
@@ -8721,7 +8811,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A14,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A14,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C14" s="24" t="n">
@@ -8740,7 +8830,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A15,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A15,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C15" s="24" t="n">
@@ -8759,7 +8849,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A16,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A16,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C16" s="24" t="n">
@@ -8778,7 +8868,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A17,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A17,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C17" s="24" t="n">
@@ -8797,7 +8887,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A18,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A18,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C18" s="24" t="n">
@@ -8816,7 +8906,7 @@
         </is>
       </c>
       <c r="B19" s="15">
-        <f>SUMIFS('Renovation Ledger'!E5:E149,'Renovation Ledger'!B5:B149,A19,'Renovation Ledger'!H5:H149,"Paid")</f>
+        <f>SUMIFS('Renovation Ledger'!E5:E151,'Renovation Ledger'!B5:B151,A19,'Renovation Ledger'!H5:H151,"Paid")</f>
         <v/>
       </c>
       <c r="C19" s="24" t="n">
@@ -9062,7 +9152,7 @@
         </is>
       </c>
       <c r="C19" s="41">
-        <f>'Renovation Ledger'!E152</f>
+        <f>'Renovation Ledger'!E154</f>
         <v/>
       </c>
     </row>
@@ -9083,7 +9173,7 @@
         </is>
       </c>
       <c r="C21" s="43">
-        <f>'Renovation Ledger'!E152-69935.92</f>
+        <f>'Renovation Ledger'!E154-69935.92</f>
         <v/>
       </c>
     </row>
@@ -9136,7 +9226,7 @@
         </is>
       </c>
       <c r="C29" s="41">
-        <f>SUMPRODUCT(('Renovation Ledger'!I5:I149&gt;"2026-06-25")*('Renovation Ledger'!H5:H149="Paid")*('Renovation Ledger'!G5:G149="Yes")*'Renovation Ledger'!E5:E149)</f>
+        <f>SUMPRODUCT(('Renovation Ledger'!I5:I151&gt;"2026-06-25")*('Renovation Ledger'!H5:H151="Paid")*('Renovation Ledger'!G5:G151="Yes")*'Renovation Ledger'!E5:E151)</f>
         <v/>
       </c>
     </row>
@@ -9154,11 +9244,11 @@
     <row r="31">
       <c r="B31" s="29" t="inlineStr">
         <is>
-          <t>Reported balance (2026-07-13)</t>
+          <t>Reported balance (2026-07-21)</t>
         </is>
       </c>
       <c r="C31" s="47" t="n">
-        <v>70000</v>
+        <v>65505</v>
       </c>
     </row>
     <row r="32">

</xml_diff>